<commit_message>
Plan workbook (8 ha, lender-sized debt) with live formulas, matching finance.py exactly; lead workbook made tranche-generic
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fz2xL1bsNgN2aY5TSjEKYu
</commit_message>
<xml_diff>
--- a/business_plan/Lead_Finance_Model.xlsx
+++ b/business_plan/Lead_Finance_Model.xlsx
@@ -75,7 +75,7 @@
     <t xml:space="preserve">Minimum real price for DSCR 1.25 (finance.py solver): flex Inputs!price until 'Lender test met' turns yes.</t>
   </si>
   <si>
-    <t xml:space="preserve">finance.py minimum price (GBP/kg)</t>
+    <t xml:space="preserve">Minimum price (GBP/kg)</t>
   </si>
   <si>
     <t xml:space="preserve">Lead finance model: inputs (blue = input)</t>
@@ -5182,127 +5182,127 @@
         <v>144</v>
       </c>
       <c r="C27" s="21" t="n">
-        <f aca="false">C11-C21-C24-C19</f>
+        <f aca="false">C11-C19-C21-C24</f>
         <v>-7800399.64070004</v>
       </c>
       <c r="D27" s="21" t="n">
-        <f aca="false">D11-D21-D24-D19</f>
+        <f aca="false">D11-D19-D21-D24</f>
         <v>547362.678010144</v>
       </c>
       <c r="E27" s="21" t="n">
-        <f aca="false">E11-E21-E24-E19</f>
+        <f aca="false">E11-E19-E21-E24</f>
         <v>1338262.97388618</v>
       </c>
       <c r="F27" s="21" t="n">
-        <f aca="false">F11-F21-F24-F19</f>
+        <f aca="false">F11-F19-F21-F24</f>
         <v>1426131.90558073</v>
       </c>
       <c r="G27" s="21" t="n">
-        <f aca="false">G11-G21-G24-G19</f>
+        <f aca="false">G11-G19-G21-G24</f>
         <v>1515686.02500787</v>
       </c>
       <c r="H27" s="21" t="n">
-        <f aca="false">H11-H21-H24-H19</f>
+        <f aca="false">H11-H19-H21-H24</f>
         <v>1607069.98475236</v>
       </c>
       <c r="I27" s="21" t="n">
-        <f aca="false">I11-I21-I24-I19</f>
+        <f aca="false">I11-I19-I21-I24</f>
         <v>1700433.77328937</v>
       </c>
       <c r="J27" s="21" t="n">
-        <f aca="false">J11-J21-J24-J19</f>
+        <f aca="false">J11-J19-J21-J24</f>
         <v>1795933.31211568</v>
       </c>
       <c r="K27" s="21" t="n">
-        <f aca="false">K11-K21-K24-K19</f>
+        <f aca="false">K11-K19-K21-K24</f>
         <v>1893731.07998771</v>
       </c>
       <c r="L27" s="21" t="n">
-        <f aca="false">L11-L21-L24-L19</f>
+        <f aca="false">L11-L19-L21-L24</f>
         <v>1993996.76701966</v>
       </c>
       <c r="M27" s="21" t="n">
-        <f aca="false">M11-M21-M24-M19</f>
+        <f aca="false">M11-M19-M21-M24</f>
         <v>1802083.8934604</v>
       </c>
       <c r="N27" s="21" t="n">
-        <f aca="false">N11-N21-N24-N19</f>
+        <f aca="false">N11-N19-N21-N24</f>
         <v>2186964.00721923</v>
       </c>
       <c r="O27" s="21" t="n">
-        <f aca="false">O11-O21-O24-O19</f>
+        <f aca="false">O11-O19-O21-O24</f>
         <v>2259907.18995085</v>
       </c>
       <c r="P27" s="21" t="n">
-        <f aca="false">P11-P21-P24-P19</f>
+        <f aca="false">P11-P19-P21-P24</f>
         <v>2333453.20931836</v>
       </c>
       <c r="Q27" s="21" t="n">
-        <f aca="false">Q11-Q21-Q24-Q19</f>
+        <f aca="false">Q11-Q19-Q21-Q24</f>
         <v>2407642.10435902</v>
       </c>
       <c r="R27" s="21" t="n">
-        <f aca="false">R11-R21-R24-R19</f>
+        <f aca="false">R11-R19-R21-R24</f>
         <v>1742832.5250947</v>
       </c>
       <c r="S27" s="21" t="n">
-        <f aca="false">S11-S21-S24-S19</f>
+        <f aca="false">S11-S19-S21-S24</f>
         <v>2518747.78432216</v>
       </c>
       <c r="T27" s="21" t="n">
-        <f aca="false">T11-T21-T24-T19</f>
+        <f aca="false">T11-T19-T21-T24</f>
         <v>2577975.80181872</v>
       </c>
       <c r="U27" s="21" t="n">
-        <f aca="false">U11-U21-U24-U19</f>
+        <f aca="false">U11-U19-U21-U24</f>
         <v>2637857.1959566</v>
       </c>
       <c r="V27" s="21" t="n">
-        <f aca="false">V11-V21-V24-V19</f>
+        <f aca="false">V11-V19-V21-V24</f>
         <v>2698436.90529116</v>
       </c>
       <c r="W27" s="21" t="n">
-        <f aca="false">W11-W21-W24-W19</f>
+        <f aca="false">W11-W19-W21-W24</f>
         <v>2082720.21120798</v>
       </c>
       <c r="X27" s="21" t="n">
-        <f aca="false">X11-X21-X24-X19</f>
+        <f aca="false">X11-X19-X21-X24</f>
         <v>2785842.48521693</v>
       </c>
       <c r="Y27" s="21" t="n">
-        <f aca="false">Y11-Y21-Y24-Y19</f>
+        <f aca="false">Y11-Y19-Y21-Y24</f>
         <v>2850938.51783982</v>
       </c>
       <c r="Z27" s="21" t="n">
-        <f aca="false">Z11-Z21-Z24-Z19</f>
+        <f aca="false">Z11-Z19-Z21-Z24</f>
         <v>2916773.72014005</v>
       </c>
       <c r="AA27" s="21" t="n">
-        <f aca="false">AA11-AA21-AA24-AA19</f>
+        <f aca="false">AA11-AA19-AA21-AA24</f>
         <v>2983396.64056969</v>
       </c>
       <c r="AB27" s="21" t="n">
-        <f aca="false">AB11-AB21-AB24-AB19</f>
+        <f aca="false">AB11-AB19-AB21-AB24</f>
         <v>1011536.63984484</v>
       </c>
       <c r="AC27" s="21" t="n">
-        <f aca="false">AC11-AC21-AC24-AC19</f>
+        <f aca="false">AC11-AC19-AC21-AC24</f>
         <v>3010687.53966325</v>
       </c>
       <c r="AD27" s="21" t="n">
-        <f aca="false">AD11-AD21-AD24-AD19</f>
+        <f aca="false">AD11-AD19-AD21-AD24</f>
         <v>3086465.27978689</v>
       </c>
       <c r="AE27" s="21" t="n">
-        <f aca="false">AE11-AE21-AE24-AE19</f>
+        <f aca="false">AE11-AE19-AE21-AE24</f>
         <v>3162824.73535318</v>
       </c>
       <c r="AF27" s="21" t="n">
-        <f aca="false">AF11-AF21-AF24-AF19</f>
+        <f aca="false">AF11-AF19-AF21-AF24</f>
         <v>3239833.57103256</v>
       </c>
       <c r="AG27" s="21" t="n">
-        <f aca="false">AG11-AG21-AG24-AG19</f>
+        <f aca="false">AG11-AG19-AG21-AG24</f>
         <v>4701770.07018299</v>
       </c>
     </row>
@@ -5593,7 +5593,7 @@
       </c>
       <c r="I30" s="21" t="n">
         <f aca="false">Inputs!$C$7*(MAX(I27,0)-I28)</f>
-        <v>83636.9249566526</v>
+        <v>83636.9249566527</v>
       </c>
       <c r="J30" s="21" t="n">
         <f aca="false">Inputs!$C$7*(MAX(J27,0)-J28)</f>

</xml_diff>